<commit_message>
Fit-Gap summary: classify all 14 BRDs with one method and widen integration detection
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Programme/FitGap/BIBS_FitGap_BRD-00_Core_Replacement_BRD_vs_OOTB_vs_Best_Practice_v1.0.xlsx
+++ b/docs/deliverables/out/Programme/FitGap/BIBS_FitGap_BRD-00_Core_Replacement_BRD_vs_OOTB_vs_Best_Practice_v1.0.xlsx
@@ -64,12 +64,12 @@
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="009E9E9E"/>
+      <color rgb="00616161"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="00616161"/>
+      <color rgb="009E9E9E"/>
       <sz val="10"/>
     </font>
     <font>
@@ -844,7 +844,7 @@
       </c>
       <c r="C22" s="12" t="inlineStr">
         <is>
-          <t>Counts of the Fit-Gap sheet; 199 rows in scope.</t>
+          <t>Counts of the Fit-Gap sheet; 197 rows in scope.</t>
         </is>
       </c>
       <c r="D22" s="12" t="n">
@@ -3831,39 +3831,39 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="12" t="inlineStr">
+      <c r="A75" s="22" t="inlineStr">
         <is>
           <t>CORE-08.02</t>
         </is>
       </c>
-      <c r="B75" s="12" t="inlineStr">
+      <c r="B75" s="22" t="inlineStr">
         <is>
           <t>FR-AC-050</t>
         </is>
       </c>
-      <c r="C75" s="12" t="inlineStr">
+      <c r="C75" s="22" t="inlineStr">
         <is>
           <t>Daily cash movement reconciliation (p.8) (umbrella BR-067); covered by BRD-5 FRBS 3.3.0</t>
         </is>
       </c>
-      <c r="D75" s="12" t="inlineStr">
-        <is>
-          <t>Black (BRD)</t>
-        </is>
-      </c>
-      <c r="E75" s="12" t="inlineStr">
-        <is>
-          <t>Extend</t>
-        </is>
-      </c>
-      <c r="F75" s="12" t="inlineStr">
+      <c r="D75" s="22" t="inlineStr">
+        <is>
+          <t>Grey (Integration)</t>
+        </is>
+      </c>
+      <c r="E75" s="22" t="inlineStr">
+        <is>
+          <t>Integration scope</t>
+        </is>
+      </c>
+      <c r="F75" s="22" t="inlineStr">
         <is>
           <t>BIL-019, ACC-011</t>
         </is>
       </c>
-      <c r="G75" s="12" t="inlineStr">
-        <is>
-          <t>Deposits in transit and bank book reports; no cashier end-of-day balancing.; Statement import (BDO, BPI, Metrobank, generic), six auto-match rules, adjustments, reconciliation statement with approval. BIBS screens: SCR-AC-14, SCR-AC-15, SCR-AC-16.</t>
+      <c r="G75" s="22" t="inlineStr">
+        <is>
+          <t>Depends on an interface with another BDO or third-party system; Integration scope. BIBS screens: SCR-AC-14, SCR-AC-15, SCR-AC-16.</t>
         </is>
       </c>
     </row>
@@ -6310,111 +6310,111 @@
       </c>
     </row>
     <row r="142">
-      <c r="A142" s="22" t="inlineStr">
+      <c r="A142" s="23" t="inlineStr">
         <is>
           <t>CORE-14.08</t>
         </is>
       </c>
-      <c r="B142" s="22" t="inlineStr">
+      <c r="B142" s="23" t="inlineStr">
         <is>
           <t>CLR-CR-02 (CRQ03)</t>
         </is>
       </c>
-      <c r="C142" s="22" t="inlineStr">
+      <c r="C142" s="23" t="inlineStr">
         <is>
           <t>Unclaimed checks safekeeping (p.10) (umbrella BR-146); covered by BRD-7</t>
         </is>
       </c>
-      <c r="D142" s="22" t="inlineStr">
+      <c r="D142" s="23" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E142" s="22" t="inlineStr">
+      <c r="E142" s="23" t="inlineStr">
         <is>
           <t>Specified in another FRS</t>
         </is>
       </c>
-      <c r="F142" s="22" t="inlineStr">
+      <c r="F142" s="23" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G142" s="22" t="inlineStr">
+      <c r="G142" s="23" t="inlineStr">
         <is>
           <t>Specified in BRD-7.</t>
         </is>
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="22" t="inlineStr">
+      <c r="A143" s="23" t="inlineStr">
         <is>
           <t>CORE-14.09</t>
         </is>
       </c>
-      <c r="B143" s="22" t="inlineStr">
+      <c r="B143" s="23" t="inlineStr">
         <is>
           <t>CLR-CR-02 (CRQ03)</t>
         </is>
       </c>
-      <c r="C143" s="22" t="inlineStr">
+      <c r="C143" s="23" t="inlineStr">
         <is>
           <t>Handover of settlement checks to Cashiering (p.10) (umbrella BR-147); covered by BRD-7</t>
         </is>
       </c>
-      <c r="D143" s="22" t="inlineStr">
+      <c r="D143" s="23" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E143" s="22" t="inlineStr">
+      <c r="E143" s="23" t="inlineStr">
         <is>
           <t>Specified in another FRS</t>
         </is>
       </c>
-      <c r="F143" s="22" t="inlineStr">
+      <c r="F143" s="23" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G143" s="22" t="inlineStr">
+      <c r="G143" s="23" t="inlineStr">
         <is>
           <t>Specified in BRD-7.</t>
         </is>
       </c>
     </row>
     <row r="144">
-      <c r="A144" s="22" t="inlineStr">
+      <c r="A144" s="23" t="inlineStr">
         <is>
           <t>CORE-14.10</t>
         </is>
       </c>
-      <c r="B144" s="22" t="inlineStr">
+      <c r="B144" s="23" t="inlineStr">
         <is>
           <t>CLR-CR-02 (CRQ03)</t>
         </is>
       </c>
-      <c r="C144" s="22" t="inlineStr">
+      <c r="C144" s="23" t="inlineStr">
         <is>
           <t>Retrieval of checks from Cashiering for release (p.10) (umbrella BR-148); covered by BRD-7</t>
         </is>
       </c>
-      <c r="D144" s="22" t="inlineStr">
+      <c r="D144" s="23" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E144" s="22" t="inlineStr">
+      <c r="E144" s="23" t="inlineStr">
         <is>
           <t>Specified in another FRS</t>
         </is>
       </c>
-      <c r="F144" s="22" t="inlineStr">
+      <c r="F144" s="23" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G144" s="22" t="inlineStr">
+      <c r="G144" s="23" t="inlineStr">
         <is>
           <t>Specified in BRD-7.</t>
         </is>
@@ -6532,370 +6532,370 @@
       </c>
     </row>
     <row r="148">
-      <c r="A148" s="22" t="inlineStr">
+      <c r="A148" s="23" t="inlineStr">
         <is>
           <t>CORE-15.01</t>
         </is>
       </c>
-      <c r="B148" s="22" t="inlineStr">
+      <c r="B148" s="23" t="inlineStr">
         <is>
           <t>Phase 2</t>
         </is>
       </c>
-      <c r="C148" s="22" t="inlineStr">
+      <c r="C148" s="23" t="inlineStr">
         <is>
           <t>Placement request initiation (p.10) (umbrella BR-153); covered by ReInsurance BRD FRID-001-FRID-010</t>
         </is>
       </c>
-      <c r="D148" s="22" t="inlineStr">
+      <c r="D148" s="23" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E148" s="22" t="inlineStr">
+      <c r="E148" s="23" t="inlineStr">
         <is>
           <t>Specified in another FRS</t>
         </is>
       </c>
-      <c r="F148" s="22" t="inlineStr">
+      <c r="F148" s="23" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G148" s="22" t="inlineStr">
+      <c r="G148" s="23" t="inlineStr">
         <is>
           <t>Specified in ReInsurance BRD FRID-001-FRID-010.</t>
         </is>
       </c>
     </row>
     <row r="149">
-      <c r="A149" s="22" t="inlineStr">
+      <c r="A149" s="23" t="inlineStr">
         <is>
           <t>CORE-15.02</t>
         </is>
       </c>
-      <c r="B149" s="22" t="inlineStr">
+      <c r="B149" s="23" t="inlineStr">
         <is>
           <t>Phase 2</t>
         </is>
       </c>
-      <c r="C149" s="22" t="inlineStr">
+      <c r="C149" s="23" t="inlineStr">
         <is>
           <t>Placement slip management (p.10) (umbrella BR-154); covered by ReInsurance BRD FRID-017-FRID-028</t>
         </is>
       </c>
-      <c r="D149" s="22" t="inlineStr">
+      <c r="D149" s="23" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E149" s="22" t="inlineStr">
+      <c r="E149" s="23" t="inlineStr">
         <is>
           <t>Specified in another FRS</t>
         </is>
       </c>
-      <c r="F149" s="22" t="inlineStr">
+      <c r="F149" s="23" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G149" s="22" t="inlineStr">
+      <c r="G149" s="23" t="inlineStr">
         <is>
           <t>Specified in ReInsurance BRD FRID-017-FRID-028.</t>
         </is>
       </c>
     </row>
     <row r="150">
-      <c r="A150" s="22" t="inlineStr">
+      <c r="A150" s="23" t="inlineStr">
         <is>
           <t>CORE-15.03</t>
         </is>
       </c>
-      <c r="B150" s="22" t="inlineStr">
+      <c r="B150" s="23" t="inlineStr">
         <is>
           <t>Phase 2</t>
         </is>
       </c>
-      <c r="C150" s="22" t="inlineStr">
+      <c r="C150" s="23" t="inlineStr">
         <is>
           <t>Statement of Account (SOA) generation (p.10) (umbrella BR-155, BR-156); covered by ReInsurance BRD FRID-033-FRID-041</t>
         </is>
       </c>
-      <c r="D150" s="22" t="inlineStr">
+      <c r="D150" s="23" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E150" s="22" t="inlineStr">
+      <c r="E150" s="23" t="inlineStr">
         <is>
           <t>Specified in another FRS</t>
         </is>
       </c>
-      <c r="F150" s="22" t="inlineStr">
+      <c r="F150" s="23" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G150" s="22" t="inlineStr">
+      <c r="G150" s="23" t="inlineStr">
         <is>
           <t>Specified in ReInsurance BRD FRID-033-FRID-041.</t>
         </is>
       </c>
     </row>
     <row r="151">
-      <c r="A151" s="22" t="inlineStr">
+      <c r="A151" s="23" t="inlineStr">
         <is>
           <t>CORE-15.04</t>
         </is>
       </c>
-      <c r="B151" s="22" t="inlineStr">
+      <c r="B151" s="23" t="inlineStr">
         <is>
           <t>Phase 2</t>
         </is>
       </c>
-      <c r="C151" s="22" t="inlineStr">
+      <c r="C151" s="23" t="inlineStr">
         <is>
           <t>Claims reporting and settlement (p.10) (umbrella BR-157); covered by ReInsurance BRD FRID-101-FRID-105</t>
         </is>
       </c>
-      <c r="D151" s="22" t="inlineStr">
+      <c r="D151" s="23" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E151" s="22" t="inlineStr">
+      <c r="E151" s="23" t="inlineStr">
         <is>
           <t>Specified in another FRS</t>
         </is>
       </c>
-      <c r="F151" s="22" t="inlineStr">
+      <c r="F151" s="23" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G151" s="22" t="inlineStr">
+      <c r="G151" s="23" t="inlineStr">
         <is>
           <t>Specified in ReInsurance BRD FRID-101-FRID-105.</t>
         </is>
       </c>
     </row>
     <row r="152">
-      <c r="A152" s="22" t="inlineStr">
+      <c r="A152" s="23" t="inlineStr">
         <is>
           <t>CORE-15.05</t>
         </is>
       </c>
-      <c r="B152" s="22" t="inlineStr">
+      <c r="B152" s="23" t="inlineStr">
         <is>
           <t>Phase 2</t>
         </is>
       </c>
-      <c r="C152" s="22" t="inlineStr">
+      <c r="C152" s="23" t="inlineStr">
         <is>
           <t>Claims payment processing (p.10) (umbrella BR-158); covered by ReInsurance BRD FRID-058-FRID-066</t>
         </is>
       </c>
-      <c r="D152" s="22" t="inlineStr">
+      <c r="D152" s="23" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E152" s="22" t="inlineStr">
+      <c r="E152" s="23" t="inlineStr">
         <is>
           <t>Specified in another FRS</t>
         </is>
       </c>
-      <c r="F152" s="22" t="inlineStr">
+      <c r="F152" s="23" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G152" s="22" t="inlineStr">
+      <c r="G152" s="23" t="inlineStr">
         <is>
           <t>Specified in ReInsurance BRD FRID-058-FRID-066.</t>
         </is>
       </c>
     </row>
     <row r="153">
-      <c r="A153" s="22" t="inlineStr">
+      <c r="A153" s="23" t="inlineStr">
         <is>
           <t>CORE-15.06</t>
         </is>
       </c>
-      <c r="B153" s="22" t="inlineStr">
+      <c r="B153" s="23" t="inlineStr">
         <is>
           <t>Phase 2</t>
         </is>
       </c>
-      <c r="C153" s="22" t="inlineStr">
+      <c r="C153" s="23" t="inlineStr">
         <is>
           <t>Direct client claims payment (p.11) (umbrella BR-159); covered by ReInsurance BRD FRID-075-FRID-082</t>
         </is>
       </c>
-      <c r="D153" s="22" t="inlineStr">
+      <c r="D153" s="23" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E153" s="22" t="inlineStr">
+      <c r="E153" s="23" t="inlineStr">
         <is>
           <t>Specified in another FRS</t>
         </is>
       </c>
-      <c r="F153" s="22" t="inlineStr">
+      <c r="F153" s="23" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G153" s="22" t="inlineStr">
+      <c r="G153" s="23" t="inlineStr">
         <is>
           <t>Specified in ReInsurance BRD FRID-075-FRID-082.</t>
         </is>
       </c>
     </row>
     <row r="154">
-      <c r="A154" s="22" t="inlineStr">
+      <c r="A154" s="23" t="inlineStr">
         <is>
           <t>CORE-15.07</t>
         </is>
       </c>
-      <c r="B154" s="22" t="inlineStr">
+      <c r="B154" s="23" t="inlineStr">
         <is>
           <t>Phase 2</t>
         </is>
       </c>
-      <c r="C154" s="22" t="inlineStr">
+      <c r="C154" s="23" t="inlineStr">
         <is>
           <t>Receive and validate file from stakeholders (capability matrix p.28); covered by ReInsurance BRD</t>
         </is>
       </c>
-      <c r="D154" s="22" t="inlineStr">
+      <c r="D154" s="23" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E154" s="22" t="inlineStr">
+      <c r="E154" s="23" t="inlineStr">
         <is>
           <t>Specified in another FRS</t>
         </is>
       </c>
-      <c r="F154" s="22" t="inlineStr">
+      <c r="F154" s="23" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G154" s="22" t="inlineStr">
+      <c r="G154" s="23" t="inlineStr">
         <is>
           <t>Specified in ReInsurance BRD.</t>
         </is>
       </c>
     </row>
     <row r="155">
-      <c r="A155" s="22" t="inlineStr">
+      <c r="A155" s="23" t="inlineStr">
         <is>
           <t>CORE-15.08</t>
         </is>
       </c>
-      <c r="B155" s="22" t="inlineStr">
+      <c r="B155" s="23" t="inlineStr">
         <is>
           <t>Phase 2</t>
         </is>
       </c>
-      <c r="C155" s="22" t="inlineStr">
+      <c r="C155" s="23" t="inlineStr">
         <is>
           <t>Notification to stakeholders (capability matrix p.28); covered by ReInsurance BRD</t>
         </is>
       </c>
-      <c r="D155" s="22" t="inlineStr">
+      <c r="D155" s="23" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E155" s="22" t="inlineStr">
+      <c r="E155" s="23" t="inlineStr">
         <is>
           <t>Specified in another FRS</t>
         </is>
       </c>
-      <c r="F155" s="22" t="inlineStr">
+      <c r="F155" s="23" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G155" s="22" t="inlineStr">
+      <c r="G155" s="23" t="inlineStr">
         <is>
           <t>Specified in ReInsurance BRD.</t>
         </is>
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="22" t="inlineStr">
+      <c r="A156" s="23" t="inlineStr">
         <is>
           <t>CORE-15.09</t>
         </is>
       </c>
-      <c r="B156" s="22" t="inlineStr">
+      <c r="B156" s="23" t="inlineStr">
         <is>
           <t>Phase 2</t>
         </is>
       </c>
-      <c r="C156" s="22" t="inlineStr">
+      <c r="C156" s="23" t="inlineStr">
         <is>
           <t>Log, audit and history for traceability (capability matrix p.28); covered by ReInsurance BRD</t>
         </is>
       </c>
-      <c r="D156" s="22" t="inlineStr">
+      <c r="D156" s="23" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E156" s="22" t="inlineStr">
+      <c r="E156" s="23" t="inlineStr">
         <is>
           <t>Specified in another FRS</t>
         </is>
       </c>
-      <c r="F156" s="22" t="inlineStr">
+      <c r="F156" s="23" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G156" s="22" t="inlineStr">
+      <c r="G156" s="23" t="inlineStr">
         <is>
           <t>Specified in ReInsurance BRD.</t>
         </is>
       </c>
     </row>
     <row r="157">
-      <c r="A157" s="22" t="inlineStr">
+      <c r="A157" s="23" t="inlineStr">
         <is>
           <t>CORE-15.10</t>
         </is>
       </c>
-      <c r="B157" s="22" t="inlineStr">
+      <c r="B157" s="23" t="inlineStr">
         <is>
           <t>Phase 2</t>
         </is>
       </c>
-      <c r="C157" s="22" t="inlineStr">
+      <c r="C157" s="23" t="inlineStr">
         <is>
           <t>Net settlement (capability matrix p.28); covered by ReInsurance BRD</t>
         </is>
       </c>
-      <c r="D157" s="22" t="inlineStr">
+      <c r="D157" s="23" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E157" s="22" t="inlineStr">
+      <c r="E157" s="23" t="inlineStr">
         <is>
           <t>Specified in another FRS</t>
         </is>
       </c>
-      <c r="F157" s="22" t="inlineStr">
+      <c r="F157" s="23" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G157" s="22" t="inlineStr">
+      <c r="G157" s="23" t="inlineStr">
         <is>
           <t>Specified in ReInsurance BRD.</t>
         </is>
@@ -8715,39 +8715,39 @@
       </c>
     </row>
     <row r="207">
-      <c r="A207" s="12" t="inlineStr">
+      <c r="A207" s="22" t="inlineStr">
         <is>
           <t>XC-11</t>
         </is>
       </c>
-      <c r="B207" s="12" t="inlineStr">
+      <c r="B207" s="22" t="inlineStr">
         <is>
           <t>FR-NB-090, FR-NB-091, FR-NB-092</t>
         </is>
       </c>
-      <c r="C207" s="12" t="inlineStr">
+      <c r="C207" s="22" t="inlineStr">
         <is>
           <t>Billing reports with premium and loan details; payment reports matched to accounts (p.15) (umbrella BR-049, BR-050); covered by BRD-1 BRNB.067, BRNB.068</t>
         </is>
       </c>
-      <c r="D207" s="12" t="inlineStr">
-        <is>
-          <t>Black (BRD)</t>
-        </is>
-      </c>
-      <c r="E207" s="12" t="inlineStr">
-        <is>
-          <t>Extend</t>
-        </is>
-      </c>
-      <c r="F207" s="12" t="inlineStr">
+      <c r="D207" s="22" t="inlineStr">
+        <is>
+          <t>Grey (Integration)</t>
+        </is>
+      </c>
+      <c r="E207" s="22" t="inlineStr">
+        <is>
+          <t>Integration scope</t>
+        </is>
+      </c>
+      <c r="F207" s="22" t="inlineStr">
         <is>
           <t>QPL-024, BIL-001, QPL-023</t>
         </is>
       </c>
-      <c r="G207" s="12" t="inlineStr">
-        <is>
-          <t>Bank statement import and matching exist; no loan billing file. A bank interface would be a change request.; Premium bill (INV-) raised on policy issue, endorsement and renewal with VAT, DST and LGT booked to their own accounts; printable and e-mailed.; No payment condition on placement; claims can be blocked while premium is unpaid. BIBS screens: SCR-NB-19, SCR-NB-21.</t>
+      <c r="G207" s="22" t="inlineStr">
+        <is>
+          <t>Depends on an interface with another BDO or third-party system; Integration scope. BIBS screens: SCR-NB-19, SCR-NB-21.</t>
         </is>
       </c>
     </row>
@@ -9011,111 +9011,111 @@
       </c>
     </row>
     <row r="215">
-      <c r="A215" s="23" t="inlineStr">
+      <c r="A215" s="22" t="inlineStr">
         <is>
           <t>XC-19</t>
         </is>
       </c>
-      <c r="B215" s="23" t="inlineStr">
+      <c r="B215" s="22" t="inlineStr">
         <is>
           <t>FR-CR-081, FR-NB-117</t>
         </is>
       </c>
-      <c r="C215" s="23" t="inlineStr">
+      <c r="C215" s="22" t="inlineStr">
         <is>
           <t>Invoice batch printing, delivery to insurers by file transfer and delivery report (daily, per insurer) (p.43); covered by None (BRNB.100.1 related)</t>
         </is>
       </c>
-      <c r="D215" s="23" t="inlineStr">
+      <c r="D215" s="22" t="inlineStr">
         <is>
           <t>Grey (Integration)</t>
         </is>
       </c>
-      <c r="E215" s="23" t="inlineStr">
+      <c r="E215" s="22" t="inlineStr">
         <is>
           <t>Integration scope</t>
         </is>
       </c>
-      <c r="F215" s="23" t="inlineStr">
+      <c r="F215" s="22" t="inlineStr">
         <is>
           <t>POL-017, INT-021</t>
         </is>
       </c>
-      <c r="G215" s="23" t="inlineStr">
+      <c r="G215" s="22" t="inlineStr">
         <is>
           <t>Depends on an interface with another BDO or third-party system; Integration scope. BIBS screens: SCR-NB-32, SCR-NB-34.</t>
         </is>
       </c>
     </row>
     <row r="216">
-      <c r="A216" s="23" t="inlineStr">
+      <c r="A216" s="22" t="inlineStr">
         <is>
           <t>XC-20</t>
         </is>
       </c>
-      <c r="B216" s="23" t="inlineStr">
+      <c r="B216" s="22" t="inlineStr">
         <is>
           <t>FR-CR-082</t>
         </is>
       </c>
-      <c r="C216" s="23" t="inlineStr">
+      <c r="C216" s="22" t="inlineStr">
         <is>
           <t>Client migration (one-time, 2020 to present) and daily midday / EOD client batches with modification report (p.43); covered by Data Migration BRD V0.03; Data Migration Handbook (BRD-13)</t>
         </is>
       </c>
-      <c r="D216" s="23" t="inlineStr">
+      <c r="D216" s="22" t="inlineStr">
         <is>
           <t>Grey (Data Migration)</t>
         </is>
       </c>
-      <c r="E216" s="23" t="inlineStr">
+      <c r="E216" s="22" t="inlineStr">
         <is>
           <t>Data Migration scope</t>
         </is>
       </c>
-      <c r="F216" s="23" t="inlineStr">
+      <c r="F216" s="22" t="inlineStr">
         <is>
           <t>CRM-016, MIG-030</t>
         </is>
       </c>
-      <c r="G216" s="23" t="inlineStr">
+      <c r="G216" s="22" t="inlineStr">
         <is>
           <t>One-time or recurring load of legacy data; Data Migration scope.</t>
         </is>
       </c>
     </row>
     <row r="217">
-      <c r="A217" s="23" t="inlineStr">
+      <c r="A217" s="22" t="inlineStr">
         <is>
           <t>XC-21</t>
         </is>
       </c>
-      <c r="B217" s="23" t="inlineStr">
+      <c r="B217" s="22" t="inlineStr">
         <is>
           <t>CLR-CR-10 (CRQ20)</t>
         </is>
       </c>
-      <c r="C217" s="23" t="inlineStr">
+      <c r="C217" s="22" t="inlineStr">
         <is>
           <t>ALeA e-mail address encoding (as needed) (p.43); covered by None</t>
         </is>
       </c>
-      <c r="D217" s="23" t="inlineStr">
+      <c r="D217" s="22" t="inlineStr">
         <is>
           <t>Grey (Integration)</t>
         </is>
       </c>
-      <c r="E217" s="23" t="inlineStr">
+      <c r="E217" s="22" t="inlineStr">
         <is>
           <t>Integration scope</t>
         </is>
       </c>
-      <c r="F217" s="23" t="inlineStr">
+      <c r="F217" s="22" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G217" s="23" t="inlineStr">
+      <c r="G217" s="22" t="inlineStr">
         <is>
           <t>Depends on an interface with another BDO or third-party system; Integration scope.</t>
         </is>
@@ -9397,7 +9397,7 @@
     <row r="2">
       <c r="A2" s="19" t="inlineStr">
         <is>
-          <t>Counts of the Fit-Gap sheet; 199 rows in scope.</t>
+          <t>Counts of the Fit-Gap sheet; 197 rows in scope.</t>
         </is>
       </c>
     </row>
@@ -9460,7 +9460,7 @@
         </is>
       </c>
       <c r="B7" s="12" t="n">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
@@ -9490,7 +9490,7 @@
         </is>
       </c>
       <c r="B9" s="12" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
@@ -9565,7 +9565,7 @@
         </is>
       </c>
       <c r="B14" s="12" t="n">
-        <v>25.1</v>
+        <v>25.4</v>
       </c>
       <c r="C14" s="12" t="inlineStr">
         <is>

</xml_diff>